<commit_message>
chore: clean repository files and finalize MarginGuard codebase
</commit_message>
<xml_diff>
--- a/data/competitor_price_tracker.xlsx
+++ b/data/competitor_price_tracker.xlsx
@@ -463,7 +463,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
@@ -505,7 +505,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Lumina Medical Spa &amp; Wellness</t>
+          <t>Serenity Skin &amp; Laser Clinic</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -515,11 +515,11 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Hydrafacial Deluxe</t>
+          <t>Clear &amp; Brilliant Laser</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>225</v>
+        <v>320</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -535,7 +535,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Lumina Medical Spa &amp; Wellness</t>
+          <t>Serenity Skin &amp; Laser Clinic</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -545,11 +545,11 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Botox Cosmetic (per unit)</t>
+          <t>Dermal Fillers (1ml)</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>13.5</v>
+        <v>650</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -565,7 +565,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lumina Medical Spa &amp; Wellness</t>
+          <t>Serenity Skin &amp; Laser Clinic</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -575,11 +575,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Full Body Laser Hair Removal</t>
+          <t>IPL Photofacial</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>299</v>
+        <v>275</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -600,16 +600,16 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Aesthetics</t>
+          <t>Facial Treatments</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Microneedling with PRP</t>
+          <t>Hydrafacial Deluxe</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>450</v>
+        <v>225</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -618,7 +618,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-09-16 20:37</t>
+          <t>2026-09-16 21:33</t>
         </is>
       </c>
     </row>
@@ -630,46 +630,46 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Aesthetics</t>
+          <t>Injectables</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Morpheus8 RF Microneedling</t>
+          <t>Botox Cosmetic (per unit)</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>750</v>
+        <v>13.5</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>session</t>
+          <t>unit</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-09-16 20:37</t>
+          <t>2026-09-16 21:33</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Serenity Skin &amp; Laser Clinic</t>
+          <t>Lumina Medical Spa &amp; Wellness</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Aesthetics</t>
+          <t>Laser &amp; Body</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Clear &amp; Brilliant Laser</t>
+          <t>Full Body Laser Hair Removal</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>320</v>
+        <v>299</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -678,28 +678,28 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-09-16 20:37</t>
+          <t>2026-09-16 21:33</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Serenity Skin &amp; Laser Clinic</t>
+          <t>Lumina Medical Spa &amp; Wellness</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Aesthetics</t>
+          <t>Skin Rejuvenation</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Dermal Fillers (1ml)</t>
+          <t>Microneedling with PRP</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>650</v>
+        <v>450</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -708,28 +708,28 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-09-16 20:37</t>
+          <t>2026-09-16 21:33</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Serenity Skin &amp; Laser Clinic</t>
+          <t>Lumina Medical Spa &amp; Wellness</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Aesthetics</t>
+          <t>Skin Rejuvenation</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>IPL Photofacial</t>
+          <t>Morpheus8 RF Microneedling</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>275</v>
+        <v>750</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -738,7 +738,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-09-16 20:37</t>
+          <t>2026-09-16 21:33</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2349,6 +2349,178 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16 16:03</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Lumina Medical Spa &amp; Wellness</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Facial Treatments</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Hydrafacial Deluxe</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>199</v>
+      </c>
+      <c r="F37" s="3" t="n">
+        <v>225</v>
+      </c>
+      <c r="G37" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>+13.1%</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>PRICE INCREASE</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-16 16:03</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Lumina Medical Spa &amp; Wellness</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Laser &amp; Body</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Full Body Laser Hair Removal</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>350</v>
+      </c>
+      <c r="F38" s="4" t="n">
+        <v>299</v>
+      </c>
+      <c r="G38" s="4" t="n">
+        <v>-51</v>
+      </c>
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t>-14.6%</t>
+        </is>
+      </c>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>PRICE DECREASE</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-16 16:03</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Lumina Medical Spa &amp; Wellness</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Skin Rejuvenation</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Morpheus8 RF Microneedling</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="inlineStr">
+        <is>
+          <t>NEW ITEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-09-16 16:03</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Lumina Medical Spa &amp; Wellness</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Facial Treatments</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Chemical Peel Standard</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>120</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>DISCONTINUED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>